<commit_message>
chore: just setup was run
</commit_message>
<xml_diff>
--- a/project/excel/dcat_4c_ap.xlsx
+++ b/project/excel/dcat_4c_ap.xlsx
@@ -1,75 +1,75 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attribution" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatalogueRecord" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checksum" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChecksumAlgorithm" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concept" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConceptScheme" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataService" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DatasetSeries" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distribution" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frequency" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifier" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kind" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LegalResource" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LicenseDocument" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinguisticSystem" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediaType" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediaTypeOrExtent" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PeriodOfTime" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProvenanceStatement" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RightsStatement" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standard" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupportiveEntity" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TimeInstant" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DefinedTerm" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResearchDataset" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnalysisDataset" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResearchCatalog" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataCreatingActivity" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataAnalysis" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EvaluatedEntity" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnalysedData" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EvaluatedActivity" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HardwareTool" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoftwareTool" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QualitativeAttribute" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuantitativeAttribute" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMRAnalysisDataset" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMRSpectralAnalysis" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMRSpectroscopy" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalReaction" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalSubstance" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalEntity" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalSample" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMRSpectrum" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Laboratory" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InChIKey" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InChi" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IUPACChemicalFormula" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SMILES" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="Activity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Agent" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Attribution" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Catalogue" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CatalogueRecord" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Checksum" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ChecksumAlgorithm" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Concept" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ConceptScheme" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DataService" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Dataset" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DatasetSeries" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Distribution" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Document" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Frequency" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Geometry" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Identifier" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Kind" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="LegalResource" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="LicenseDocument" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="LinguisticSystem" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Location" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="MediaType" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="MediaTypeOrExtent" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="PeriodOfTime" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Policy" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="ProvenanceStatement" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Relationship" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Resource" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="RightsStatement" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Role" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Standard" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="SupportiveEntity" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="TimeInstant" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="DefinedTerm" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="ResearchDataset" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="AnalysisDataset" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="ResearchCatalog" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="DataCreatingActivity" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="DataAnalysis" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="EvaluatedEntity" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="AnalysedData" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="EvaluatedActivity" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Tool" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="HardwareTool" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="SoftwareTool" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="Environment" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="Plan" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="QualitativeAttribute" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="QuantitativeAttribute" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="NMRAnalysisDataset" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="NMRSpectralAnalysis" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="NMRSpectroscopy" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="ChemicalReaction" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="ChemicalSubstance" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="ChemicalEntity" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="ChemicalSample" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="NMRSpectrum" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="Laboratory" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="InChIKey" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="InChi" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="IUPACChemicalFormula" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="SMILES" sheetId="63" state="visible" r:id="rId63"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>